<commit_message>
Merge corrected labels for the 19 truncated GPT-5.5 SDXL/FLUX responses
The released SDXL/FLUX disagreement-prediction files still held 19 mid-word-truncated
"FA" responses that the letter (R1 Comment 7) says were corrected. Their corrected
labels (all FAKE) and token counts from the bugfix_reruns batch are now merged in.
No reported accuracy changes: SDXL/FLUX GPT-5.5 accuracy comes from the uniform run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results/paper_results.xlsx
+++ b/paper_results/paper_results.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-21T23:49:29+00:00</t>
+          <t>2026-10-21T23:50:53+00:00</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>f992a3048f974b4696bf52fe0f1b433dd3548b41</t>
+          <t>4c1408f3d9b0c461b039c9343e4d77f1dc2dbd27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reframe C4 around the gated cascade; add verified pricing URL
The cascade's gain under deployment shift holds with either routing signal: with
GPT-5.5, confidence routing gains 3.6-7.7 points over the stale probe vs 3.4-7.9 for
disagreement. C4, the confidence-routing discussion, the RQ2 conclusion and the R1
Comment 8 response now present the gated cascade as the contribution and disagreement
as the no-setup default that also shows which detector is failing; they no longer
compare signal accuracy. The new range is an audited inline number.

pricing_url.txt records the OpenAI pricing page (verified 2026-10-22 to list gpt-5.5
Batch at $2.50/$15.00 per 1M tokens), and the bib entry now carries the URL.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results/paper_results.xlsx
+++ b/paper_results/paper_results.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-22T01:40:09+00:00</t>
+          <t>2026-10-22T01:52:41+00:00</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>205eb2de32f0e5b0b0c6550ac7fd7c82c0ba8d88</t>
+          <t>d61af0ded7493f5ad939ef3695aa77dab3244031</t>
         </is>
       </c>
     </row>
@@ -23942,7 +23942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24176,22 +24176,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abstract, C3</t>
+          <t>V.C confidence routing</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>up to 7.9 percentage points</t>
+          <t>by 3.6--7.7 points across the</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>tab_e8_cascade.gain_gpt55 (max)</t>
+          <t>tab_confidence_routing (val_tau, semantic) - stale</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>up to 7.9 percentage points</t>
+          <t>by 3.6--7.7 points across the</t>
         </is>
       </c>
       <c r="E9" t="b">
@@ -24204,22 +24204,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Abstract, VI.J, Fig. D</t>
+          <t>Abstract, C3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>42--51\% of</t>
+          <t>up to 7.9 percentage points</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>tab_cost_accuracy_tradeoff.cascade_cost_frac_of_uniform</t>
+          <t>tab_e8_cascade.gain_gpt55 (max)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>42--51\% of</t>
+          <t>up to 7.9 percentage points</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -24232,22 +24232,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>VI.J, Fig. cost_accuracy</t>
+          <t>Abstract, VI.J, Fig. D</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>36--42\%</t>
+          <t>42--51\% of</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>tab_cost_accuracy_tradeoff.esc_rate</t>
+          <t>tab_cost_accuracy_tradeoff.cascade_cost_frac_of_uniform</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>36--42\%</t>
+          <t>42--51\% of</t>
         </is>
       </c>
       <c r="E11" t="b">
@@ -24260,22 +24260,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>VI.J, Fig. cost_accuracy</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>invocations by 58--64\%</t>
+          <t>36--42\%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1 - tab_cost_accuracy_tradeoff.esc_rate</t>
+          <t>tab_cost_accuracy_tradeoff.esc_rate</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>invocations by 58--64\%</t>
+          <t>36--42\%</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -24288,22 +24288,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>VI.J</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>dollar cost by 49--58\%</t>
+          <t>invocations by 58--64\%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>tab_cost_accuracy_tradeoff.cost_saved_vs_uniform_pct</t>
+          <t>1 - tab_cost_accuracy_tradeoff.esc_rate</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>dollar cost by 49--58\%</t>
+          <t>invocations by 58--64\%</t>
         </is>
       </c>
       <c r="E13" t="b">
@@ -24316,22 +24316,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>VI.J</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>97--100\%</t>
+          <t>dollar cost by 49--58\%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>tab_cost_accuracy_tradeoff.uniform_acc</t>
+          <t>tab_cost_accuracy_tradeoff.cost_saved_vs_uniform_pct</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>97--100\%</t>
+          <t>dollar cost by 49--58\%</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -24344,22 +24344,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>VI.J</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Uniform escalation reaches 99.6\%</t>
+          <t>97--100\%</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>tab_cost_accuracy_tradeoff.uniform_acc (SDXL)</t>
+          <t>tab_cost_accuracy_tradeoff.uniform_acc</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Uniform escalation reaches 99.6\%</t>
+          <t>97--100\%</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -24377,17 +24377,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>accuracy on SDXL and 97.1\% on FLUX</t>
+          <t>Uniform escalation reaches 99.6\%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>tab_cost_accuracy_tradeoff.uniform_acc (FLUX)</t>
+          <t>tab_cost_accuracy_tradeoff.uniform_acc (SDXL)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>accuracy on SDXL and 97.1\% on FLUX</t>
+          <t>Uniform escalation reaches 99.6\%</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -24405,17 +24405,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>3.0 to 7.8 percentage points</t>
+          <t>accuracy on SDXL and 97.1\% on FLUX</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>tab_cost_accuracy_tradeoff.gap_to_uniform</t>
+          <t>tab_cost_accuracy_tradeoff.uniform_acc (FLUX)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3.0 to 7.8 percentage points</t>
+          <t>accuracy on SDXL and 97.1\% on FLUX</t>
         </is>
       </c>
       <c r="E17" t="b">
@@ -24428,22 +24428,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>VI.J</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>21 of 33 eligible configurations at $N=100$ and 25 of 33 at $N=200$</t>
+          <t>3.0 to 7.8 percentage points</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>tab_gate_holdout (sig, &gt;=0.9)</t>
+          <t>tab_cost_accuracy_tradeoff.gap_to_uniform</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>21 of 33 eligible configurations at $N=100$ and 25 of 33 at $N=200$</t>
+          <t>3.0 to 7.8 percentage points</t>
         </is>
       </c>
       <c r="E18" t="b">
@@ -24456,22 +24456,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>VI.I.1</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>(7.3\% vs.\ 0.3\% at $N{=}50$)</t>
+          <t>21 of 33 eligible configurations at $N=100$ and 25 of 33 at $N=200$</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>tab_gate_holdout harmful rates at N=50</t>
+          <t>tab_gate_holdout (sig, &gt;=0.9)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>(7.3\% vs.\ 0.3\% at $N{=}50$)</t>
+          <t>21 of 33 eligible configurations at $N=100$ and 25 of 33 at $N=200$</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -24484,22 +24484,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>V (confidence routing)</t>
+          <t>VI.I.1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>more than 1.7 points less accurate</t>
+          <t>(7.3\% vs.\ 0.3\% at $N{=}50$)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>tab_confidence_routing (max conf - dis)</t>
+          <t>tab_gate_holdout harmful rates at N=50</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>more than 1.7 points less accurate</t>
+          <t>(7.3\% vs.\ 0.3\% at $N{=}50$)</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -24512,28 +24512,56 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>V (confidence routing)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>more than 1.7 points less accurate</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>tab_confidence_routing (max conf - dis)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>more than 1.7 points less accurate</t>
+        </is>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>V.B.1</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>The six configurations that clear</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>tab_baselines.clears_best_cheap</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>The six configurations that clear</t>
         </is>
       </c>
-      <c r="E21" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" t="b">
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Consistency pass: align claims with current results
Four statements contradicted current results. C4 and the RQ2 conclusion called
disagreement "the dominant routing signal" outright; it is dominant only among the
learned classifier's inputs. The intro credited it with "requiring no calibration"; it
needs no threshold or probability outputs. RQ3 said escalation fails under
cross-family transfer; it fails in five of six pairings (BigGAN->GenBuster is a small
gain).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results/paper_results.xlsx
+++ b/paper_results/paper_results.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-22T01:52:41+00:00</t>
+          <t>2026-10-22T01:57:02+00:00</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>d61af0ded7493f5ad939ef3695aa77dab3244031</t>
+          <t>19a467fd416f268d5893fcd5d8dd53ee317716bb</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
256 px size-matched control: GPT-5.5 + cascade results
All 7,315 images labeled by GPT-5.5 at 256x256 (Batch tier; 3,757 requests
resubmitted after a credit-exhaustion failure; 0 invalid). input_tokens =
119 for every image in both classes. Cost $25.52.

tab_e8_cascade_sizematched now has original / 512 px / 256 px. At 256 px,
where both classes are downscaled, the stale FFT probe largely recovers
(SDXL 60.0%, FLUX 54.7%; 49.3%/45.2% at 512 px), so the 512 px FFT collapse
was mostly an artifact of upscaling 96% of the reals. Cascade gain over the
stale probe stays significant in all four cells, and disagreement routing
beats random routing at the same rate in three of four (FLUX/DINOv2 n.s.).

Full regeneration: existing tables unchanged, audit 0 mismatches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_results/paper_results.xlsx
+++ b/paper_results/paper_results.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-22T20:28:55+00:00</t>
+          <t>2026-10-22T22:24:31+00:00</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bce1e4a90886722757cc6940c2d6dbcf5eee3001</t>
+          <t>5022f9b2a6fd8595dd6fbf199a1f3d7fa63dfbd6</t>
         </is>
       </c>
     </row>
@@ -23944,7 +23944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH9"/>
+  <dimension ref="A1:AH13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25013,6 +25013,454 @@
       </c>
       <c r="AH9" t="n">
         <v>350</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sizematched256</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SDXL</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SigLIP2</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.83975</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.60025</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1636</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.409</v>
+      </c>
+      <c r="K10" t="n">
+        <v>636</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.9669926650366748</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>StaleSigLIP2</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>0.7927872860635696</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.1742053789731052</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.1528117359413204</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.1955990220048899</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.911</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.07125000000000004</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.06225000000000003</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.08050000000000002</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.89292</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0.01808</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.0116244875</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.024737525</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.96975</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.4021391099043026</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0.9495</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0.9339622641509434</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0.988</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>119</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sizematched256</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SDXL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DINOv2</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.8505</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.60025</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1623</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.40575</v>
+      </c>
+      <c r="K11" t="n">
+        <v>591</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1032</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.9673444239063462</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>StaleDINOv2</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>0.8083795440542206</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.1589648798521256</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.1380160197165743</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.1799137399876771</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0.915</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.0645</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.05574999999999997</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.07324999999999993</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.8988856874999999</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0.0161143125</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.009642803124999995</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.0225855625</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.96975</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.3921074910482635</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0.9495</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0.9306260575296108</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0.9883720930232558</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>119</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sizematched256</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SigLIP2</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.8715000000000001</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.547</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1874</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.4685</v>
+      </c>
+      <c r="K12" t="n">
+        <v>681</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1193</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.9290288153681964</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>StaleSigLIP2</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>0.8463180362860192</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.08271077908217717</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.06350053361792962</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.1019210245464248</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.91025</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0.03874999999999995</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.02975000000000005</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.04774999999999996</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.902421</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0.007828999999999999</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0.001736278124999999</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0.01403175</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>0.4694211917395132</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>0.9505</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>0.9245</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>0.9295154185022027</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>0.9287510477787091</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>119</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sizematched256</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DINOv2</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.81725</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.547</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1767</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.44175</v>
+      </c>
+      <c r="K13" t="n">
+        <v>630</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1137</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.9349179400113187</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>StaleDINOv2</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>0.8058856819468024</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.1290322580645162</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.1080928126768533</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.1499717034521788</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0.87425</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.05699999999999994</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.04749999999999999</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.06674999999999998</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.8703704375000001</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0.003879562500000002</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>-0.003051279687499998</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0.01101425</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>0.4455125649693514</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>0.9505</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>0.9245</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>0.9380952380952381</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0.9331574318381706</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>119</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>